<commit_message>
minor edits for tutors
</commit_message>
<xml_diff>
--- a/teams-and-rosters/CS320-Sp25-Teams.xlsx
+++ b/teams-and-rosters/CS320-Sp25-Teams.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2025\teams-and-rosters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE7408A-8B73-4A55-B007-D747DF2937F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F48E11D-E46B-48CD-BB71-13552A1FC9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1335" yWindow="630" windowWidth="15405" windowHeight="14730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -742,7 +755,7 @@
       <c r="E5" s="18"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="2:6" s="2" customFormat="1" ht="80.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" s="2" customFormat="1" ht="86.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
         <v>8</v>
       </c>
@@ -831,7 +844,7 @@
       <c r="E14" s="18"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" ht="48.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" ht="58.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12" t="s">
         <v>10</v>
       </c>

</xml_diff>